<commit_message>
espectros del 2023 organizados
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2023.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2023.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,7 +605,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Agosto 29-2023</t>
+          <t>Agosto 28-2023</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -619,34 +619,34 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6562.228</v>
+        <v>6562.267</v>
       </c>
       <c r="E5" t="n">
-        <v>-8.899999999999999e-05</v>
+        <v>-8.3e-05</v>
       </c>
       <c r="F5" t="n">
-        <v>-26.69</v>
+        <v>-24.9</v>
       </c>
       <c r="G5" t="n">
-        <v>-56.07</v>
+        <v>-54.28</v>
       </c>
       <c r="H5" t="n">
-        <v>-54.82</v>
+        <v>-54.09</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2542</v>
+        <v>0.35</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9350000000000001</v>
+        <v>1.054</v>
       </c>
       <c r="K5" t="n">
-        <v>0.3288</v>
+        <v>0.5024999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Agosto 29-2023</t>
+          <t>Agosto 28-2023</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -660,34 +660,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6563.038</v>
+        <v>6563.002</v>
       </c>
       <c r="E6" t="n">
-        <v>3.4e-05</v>
+        <v>2.9e-05</v>
       </c>
       <c r="F6" t="n">
-        <v>10.32</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>-19.06</v>
+        <v>-20.68</v>
       </c>
       <c r="H6" t="n">
-        <v>-17.81</v>
+        <v>-20.49</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8124</v>
+        <v>0.917</v>
       </c>
       <c r="J6" t="n">
-        <v>1.095</v>
+        <v>1.128</v>
       </c>
       <c r="K6" t="n">
-        <v>0.9766</v>
+        <v>1.1508</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Agosto 29-2023</t>
+          <t>Agosto 28-2023</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -701,34 +701,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6564.013</v>
+        <v>6564.036</v>
       </c>
       <c r="E7" t="n">
-        <v>9.399999999999999e-05</v>
+        <v>9.7e-05</v>
       </c>
       <c r="F7" t="n">
-        <v>28.13</v>
+        <v>29.19</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.25</v>
+        <v>-0.19</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5497</v>
+        <v>0.5424</v>
       </c>
       <c r="J7" t="n">
-        <v>1.026</v>
+        <v>0.877</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6535</v>
+        <v>0.5579</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Septiembre 01-2023</t>
+          <t>Agosto 29-2023</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -742,34 +742,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6562.174</v>
+        <v>6562.228</v>
       </c>
       <c r="E8" t="n">
-        <v>-9.7e-05</v>
+        <v>-8.899999999999999e-05</v>
       </c>
       <c r="F8" t="n">
-        <v>-29.16</v>
+        <v>-26.69</v>
       </c>
       <c r="G8" t="n">
-        <v>-58.77</v>
+        <v>-56.23</v>
       </c>
       <c r="H8" t="n">
-        <v>-57.85</v>
+        <v>-54.82</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2506</v>
+        <v>0.2542</v>
       </c>
       <c r="J8" t="n">
-        <v>0.904</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3189</v>
+        <v>0.3288</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Septiembre 01-2023</t>
+          <t>Agosto 29-2023</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -783,34 +783,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6563.021</v>
+        <v>6563.038</v>
       </c>
       <c r="E9" t="n">
-        <v>3.2e-05</v>
+        <v>3.4e-05</v>
       </c>
       <c r="F9" t="n">
-        <v>9.539999999999999</v>
+        <v>10.32</v>
       </c>
       <c r="G9" t="n">
-        <v>-20.07</v>
+        <v>-19.22</v>
       </c>
       <c r="H9" t="n">
-        <v>-19.15</v>
+        <v>-17.81</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8598</v>
+        <v>0.8124</v>
       </c>
       <c r="J9" t="n">
-        <v>1.099</v>
+        <v>1.095</v>
       </c>
       <c r="K9" t="n">
-        <v>1.0472</v>
+        <v>0.9766</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Septiembre 01-2023</t>
+          <t>Agosto 29-2023</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -824,39 +824,39 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6564.025</v>
+        <v>6564.013</v>
       </c>
       <c r="E10" t="n">
-        <v>9.6e-05</v>
+        <v>9.399999999999999e-05</v>
       </c>
       <c r="F10" t="n">
-        <v>28.69</v>
+        <v>28.13</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.92</v>
+        <v>-1.42</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5447</v>
+        <v>0.5497</v>
       </c>
       <c r="J10" t="n">
-        <v>0.9330000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5917</v>
+        <v>0.6535</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Septiembre 08-2023</t>
+          <t>Septiembre 01-2023</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Estrella</t>
+          <t>Tierra</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -865,37 +865,39 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6561.525</v>
+        <v>6562.174</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.000196</v>
+        <v>-9.7e-05</v>
       </c>
       <c r="F11" t="n">
+        <v>-29.16</v>
+      </c>
+      <c r="G11" t="n">
         <v>-58.77</v>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>-57.41</v>
+        <v>-57.85</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2286</v>
+        <v>0.2506</v>
       </c>
       <c r="J11" t="n">
-        <v>0.896</v>
+        <v>0.904</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2855</v>
+        <v>0.3189</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Septiembre 08-2023</t>
+          <t>Septiembre 01-2023</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Estrella</t>
+          <t>Tierra</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -904,37 +906,39 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6562.395</v>
+        <v>6563.021</v>
       </c>
       <c r="E12" t="n">
-        <v>-6.4e-05</v>
+        <v>3.2e-05</v>
       </c>
       <c r="F12" t="n">
-        <v>-19.04</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+        <v>9.539999999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-20.07</v>
+      </c>
       <c r="H12" t="n">
-        <v>-17.68</v>
+        <v>-19.15</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8552</v>
+        <v>0.8598</v>
       </c>
       <c r="J12" t="n">
-        <v>1.081</v>
+        <v>1.099</v>
       </c>
       <c r="K12" t="n">
-        <v>1.0129</v>
+        <v>1.0472</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Septiembre 08-2023</t>
+          <t>Septiembre 01-2023</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Estrella</t>
+          <t>Tierra</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -943,32 +947,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6563.367</v>
+        <v>6564.025</v>
       </c>
       <c r="E13" t="n">
-        <v>-5e-06</v>
+        <v>9.6e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>-1.35</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+        <v>28.69</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-0.92</v>
+      </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0.5511</v>
+        <v>0.5447</v>
       </c>
       <c r="J13" t="n">
-        <v>0.93</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>0.5895</v>
+        <v>0.5917</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Octubre 12-2023</t>
+          <t>Septiembre 08-2023</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -982,34 +988,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6562.189</v>
+        <v>6562.204</v>
       </c>
       <c r="E14" t="n">
-        <v>-9.500000000000001e-05</v>
+        <v>-9.3e-05</v>
       </c>
       <c r="F14" t="n">
-        <v>-28.46</v>
+        <v>-27.78</v>
       </c>
       <c r="G14" t="n">
-        <v>-51.51</v>
+        <v>-57.29</v>
       </c>
       <c r="H14" t="n">
-        <v>-50.7</v>
+        <v>-58.44</v>
       </c>
       <c r="I14" t="n">
-        <v>0.5562</v>
+        <v>0.227</v>
       </c>
       <c r="J14" t="n">
-        <v>1.075</v>
+        <v>0.896</v>
       </c>
       <c r="K14" t="n">
-        <v>0.8108</v>
+        <v>0.2835</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Octubre 12-2023</t>
+          <t>Septiembre 08-2023</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1023,34 +1029,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6562.799</v>
+        <v>6563.082</v>
       </c>
       <c r="E15" t="n">
-        <v>-2e-06</v>
+        <v>4.1e-05</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.58</v>
+        <v>12.32</v>
       </c>
       <c r="G15" t="n">
-        <v>-23.63</v>
+        <v>-17.19</v>
       </c>
       <c r="H15" t="n">
-        <v>-22.81</v>
+        <v>-18.34</v>
       </c>
       <c r="I15" t="n">
-        <v>0.9992</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>1.17</v>
+        <v>1.087</v>
       </c>
       <c r="K15" t="n">
-        <v>1.3003</v>
+        <v>1.0237</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Octubre 12-2023</t>
+          <t>Septiembre 08-2023</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1064,34 +1070,34 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6563.884</v>
+        <v>6564.068</v>
       </c>
       <c r="E16" t="n">
-        <v>7.4e-05</v>
+        <v>0.000102</v>
       </c>
       <c r="F16" t="n">
-        <v>22.23</v>
+        <v>30.66</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.82</v>
+        <v>1.16</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0.5427999999999999</v>
+        <v>0.5514</v>
       </c>
       <c r="J16" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>0.6001</v>
+        <v>0.5905</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Octubre 19-2023</t>
+          <t>Octubre 12-2023</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1105,34 +1111,34 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6562.118</v>
+        <v>6562.189</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.000106</v>
+        <v>-9.500000000000001e-05</v>
       </c>
       <c r="F17" t="n">
-        <v>-31.68</v>
+        <v>-28.46</v>
       </c>
       <c r="G17" t="n">
-        <v>-52.29</v>
+        <v>-51.51</v>
       </c>
       <c r="H17" t="n">
-        <v>-54.13</v>
+        <v>-50.7</v>
       </c>
       <c r="I17" t="n">
-        <v>0.3735</v>
+        <v>0.5562</v>
       </c>
       <c r="J17" t="n">
-        <v>1.025</v>
+        <v>1.075</v>
       </c>
       <c r="K17" t="n">
-        <v>0.5181</v>
+        <v>0.8108</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Octubre 19-2023</t>
+          <t>Octubre 12-2023</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1146,34 +1152,34 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6562.88</v>
+        <v>6562.799</v>
       </c>
       <c r="E18" t="n">
-        <v>1e-05</v>
+        <v>-2e-06</v>
       </c>
       <c r="F18" t="n">
-        <v>3.11</v>
+        <v>-0.58</v>
       </c>
       <c r="G18" t="n">
-        <v>-17.5</v>
+        <v>-23.63</v>
       </c>
       <c r="H18" t="n">
-        <v>-19.34</v>
+        <v>-22.81</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8482</v>
+        <v>0.9992</v>
       </c>
       <c r="J18" t="n">
-        <v>1.113</v>
+        <v>1.17</v>
       </c>
       <c r="K18" t="n">
-        <v>1.0368</v>
+        <v>1.3003</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Octubre 19-2023</t>
+          <t>Octubre 12-2023</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1187,27 +1193,150 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6563.888</v>
+        <v>6563.884</v>
       </c>
       <c r="E19" t="n">
-        <v>7.499999999999999e-05</v>
+        <v>7.4e-05</v>
       </c>
       <c r="F19" t="n">
-        <v>22.45</v>
+        <v>22.23</v>
       </c>
       <c r="G19" t="n">
-        <v>1.84</v>
+        <v>-0.82</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
+        <v>0.5427999999999999</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.6001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Octubre 19-2023</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tierra</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>6562.118</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-0.000106</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-31.68</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-52.29</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-54.13</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.3735</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.5181</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Octubre 19-2023</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tierra</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>6562.88</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-17.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-19.34</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.8482</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1.113</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1.0368</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Octubre 19-2023</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Tierra</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>6563.888</v>
+      </c>
+      <c r="E22" t="n">
+        <v>7.499999999999999e-05</v>
+      </c>
+      <c r="F22" t="n">
+        <v>22.45</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
         <v>0.5496</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J22" t="n">
         <v>1.041</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K22" t="n">
         <v>0.6692</v>
       </c>
     </row>

</xml_diff>